<commit_message>
Finish incorporating helper package files
</commit_message>
<xml_diff>
--- a/inst/extdata/CASTool_InputCheck.xlsx
+++ b/inst/extdata/CASTool_InputCheck.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lnaslund\Documents\CASTool_Data\20250711_FinalInputDataFormat\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{84885A33-EFE6-4B05-AC6E-0A1860C916F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A9C2C67-DEB0-44DA-BE56-43987F2E70F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{C3CC5D38-EA26-4306-AA8F-FFA0E248C533}"/>
   </bookViews>
@@ -18,9 +18,9 @@
     <sheet name="paired" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">data!$A$1:$G$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">data!$A$1:$G$23</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0" concurrentManualCount="4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="124">
   <si>
     <t>Object</t>
   </si>
@@ -163,12 +163,6 @@
     <t>required</t>
   </si>
   <si>
-    <t>optional</t>
-  </si>
-  <si>
-    <t>contingent, site</t>
-  </si>
-  <si>
     <t>contingent, bc</t>
   </si>
   <si>
@@ -262,12 +256,6 @@
     <t>fn.fish.MT</t>
   </si>
   <si>
-    <t>fn.outline</t>
-  </si>
-  <si>
-    <t>STATE.shp</t>
-  </si>
-  <si>
     <t>fn.meas.data</t>
   </si>
   <si>
@@ -389,6 +377,42 @@
   </si>
   <si>
     <t>MetricName</t>
+  </si>
+  <si>
+    <t>boundary</t>
+  </si>
+  <si>
+    <t>fn.boundary</t>
+  </si>
+  <si>
+    <t>regional boundary</t>
+  </si>
+  <si>
+    <t>contigent, helperImport</t>
+  </si>
+  <si>
+    <t>fn.reaches</t>
+  </si>
+  <si>
+    <t>fn.cluster.graphic</t>
+  </si>
+  <si>
+    <t>reaches</t>
+  </si>
+  <si>
+    <t>contingent, helperImport</t>
+  </si>
+  <si>
+    <t>cluster_graphic</t>
+  </si>
+  <si>
+    <t>NHDPlusV2 reaches in boundary</t>
+  </si>
+  <si>
+    <t>cluster graphic</t>
+  </si>
+  <si>
+    <t>geometry</t>
   </si>
 </sst>
 </file>
@@ -791,13 +815,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>49</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -805,15 +829,15 @@
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="90" x14ac:dyDescent="0.25">
@@ -821,10 +845,10 @@
         <v>38</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -832,10 +856,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -852,7 +876,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BA5018B-B8C5-4E07-A0CB-63785AE486B0}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -872,7 +896,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>38</v>
@@ -881,10 +905,10 @@
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -895,7 +919,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D2" t="s">
         <v>39</v>
@@ -907,7 +931,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -918,56 +942,56 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D3" t="s">
         <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="G3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>76</v>
       </c>
       <c r="C4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D4" t="s">
-        <v>41</v>
+        <v>77</v>
       </c>
       <c r="E4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F5" t="s">
         <v>93</v>
@@ -975,404 +999,438 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C6" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D6" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="E6" t="s">
-        <v>43</v>
+        <v>83</v>
       </c>
       <c r="F6" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C7" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E7" t="s">
-        <v>87</v>
+        <v>37</v>
       </c>
       <c r="F7" t="s">
         <v>94</v>
       </c>
+      <c r="G7" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C8" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E8" t="s">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="F8" t="s">
-        <v>98</v>
-      </c>
-      <c r="G8" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E9" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="F9" t="s">
-        <v>94</v>
+        <v>95</v>
+      </c>
+      <c r="G9" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D10" t="s">
-        <v>65</v>
-      </c>
-      <c r="E10" t="s">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="F10" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="G10" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>80</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
         <v>110</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>64</v>
+      </c>
+      <c r="E11" t="s">
+        <v>100</v>
       </c>
       <c r="F11" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="G11" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C12" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="D12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E12" t="s">
-        <v>104</v>
+        <v>43</v>
       </c>
       <c r="F12" t="s">
-        <v>100</v>
-      </c>
-      <c r="G12" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>70</v>
+        <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E13" t="s">
         <v>45</v>
       </c>
       <c r="F13" t="s">
-        <v>95</v>
+        <v>97</v>
+      </c>
+      <c r="G13" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C14" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F14" t="s">
-        <v>101</v>
-      </c>
-      <c r="G14" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D15" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E15" t="s">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="F15" t="s">
-        <v>115</v>
+        <v>96</v>
+      </c>
+      <c r="G15" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="C16" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="D16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E16" t="s">
-        <v>104</v>
+        <v>43</v>
       </c>
       <c r="F16" t="s">
-        <v>100</v>
-      </c>
-      <c r="G16" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E17" t="s">
         <v>45</v>
       </c>
       <c r="F17" t="s">
-        <v>95</v>
+        <v>97</v>
+      </c>
+      <c r="G17" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C18" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F18" t="s">
-        <v>101</v>
-      </c>
-      <c r="G18" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B19" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C19" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D19" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E19" t="s">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="F19" t="s">
-        <v>115</v>
+        <v>96</v>
+      </c>
+      <c r="G19" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="C20" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="D20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E20" t="s">
-        <v>104</v>
+        <v>43</v>
       </c>
       <c r="F20" t="s">
-        <v>100</v>
-      </c>
-      <c r="G20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B21" t="s">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="C21" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E21" t="s">
         <v>45</v>
       </c>
       <c r="F21" t="s">
-        <v>95</v>
+        <v>97</v>
+      </c>
+      <c r="G21" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C22" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E22" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F22" t="s">
-        <v>101</v>
-      </c>
-      <c r="G22" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>112</v>
       </c>
       <c r="B23" t="s">
-        <v>36</v>
+        <v>113</v>
       </c>
       <c r="C23" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D23" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="E23" t="s">
-        <v>48</v>
-      </c>
-      <c r="F23" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>118</v>
       </c>
       <c r="B24" t="s">
-        <v>73</v>
+        <v>116</v>
       </c>
       <c r="C24" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="D24" t="s">
-        <v>40</v>
+        <v>119</v>
+      </c>
+      <c r="E24" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" t="s">
+        <v>103</v>
+      </c>
+      <c r="D25" t="s">
+        <v>119</v>
+      </c>
+      <c r="E25" t="s">
+        <v>44</v>
+      </c>
+      <c r="F25" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>120</v>
+      </c>
+      <c r="B26" t="s">
+        <v>117</v>
+      </c>
+      <c r="C26" t="s">
+        <v>122</v>
+      </c>
+      <c r="D26" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G24" xr:uid="{7BA5018B-B8C5-4E07-A0CB-63785AE486B0}"/>
+  <autoFilter ref="A1:G23" xr:uid="{7BA5018B-B8C5-4E07-A0CB-63785AE486B0}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1388,10 +1446,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C1" t="s">
         <v>38</v>
@@ -1399,35 +1457,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1438,7 +1496,7 @@
         <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1449,7 +1507,7 @@
         <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1460,7 +1518,7 @@
         <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1468,10 +1526,10 @@
         <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1479,10 +1537,10 @@
         <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1490,10 +1548,10 @@
         <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix WSStressor comid filtering, remove ClusterID as required data_WSStressor column, add flexibility for class for some columns
</commit_message>
<xml_diff>
--- a/inst/extdata/CASTool_InputCheck.xlsx
+++ b/inst/extdata/CASTool_InputCheck.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lnaslund\Documents\CASTool_Data\20250711_FinalInputDataFormat\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lnaslund\Documents\CASTfxn_AnnFinal\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A9C2C67-DEB0-44DA-BE56-43987F2E70F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8CC49F8-D55B-4B24-8762-EA58D58F1E5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{C3CC5D38-EA26-4306-AA8F-FFA0E248C533}"/>
+    <workbookView xWindow="-25320" yWindow="-2070" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{C3CC5D38-EA26-4306-AA8F-FFA0E248C533}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="2" r:id="rId1"/>
@@ -166,9 +166,6 @@
     <t>contingent, bc</t>
   </si>
   <si>
-    <t>COMID, ClusterID, StreamCatVar, WatershedValue, Year</t>
-  </si>
-  <si>
     <t>StreamCatVar, Label</t>
   </si>
   <si>
@@ -413,6 +410,9 @@
   </si>
   <si>
     <t>geometry</t>
+  </si>
+  <si>
+    <t>COMID, StreamCatVar, WatershedValue, Year</t>
   </si>
 </sst>
 </file>
@@ -815,13 +815,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -829,15 +829,15 @@
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="90" x14ac:dyDescent="0.25">
@@ -845,10 +845,10 @@
         <v>38</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -856,10 +856,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>54</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -896,7 +896,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>38</v>
@@ -905,10 +905,10 @@
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -919,7 +919,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D2" t="s">
         <v>39</v>
@@ -931,7 +931,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -942,19 +942,19 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D3" t="s">
         <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -962,19 +962,19 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" t="s">
         <v>76</v>
       </c>
-      <c r="C4" t="s">
-        <v>104</v>
-      </c>
-      <c r="D4" t="s">
-        <v>77</v>
-      </c>
       <c r="E4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -982,19 +982,19 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E5" t="s">
-        <v>41</v>
+        <v>123</v>
       </c>
       <c r="F5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1002,19 +1002,19 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1022,22 +1022,22 @@
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E7" t="s">
         <v>37</v>
       </c>
       <c r="F7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1045,19 +1045,19 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1065,22 +1065,22 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1091,59 +1091,59 @@
         <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D10" t="s">
         <v>40</v>
       </c>
       <c r="F10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B11" t="s">
         <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1154,19 +1154,19 @@
         <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1177,16 +1177,16 @@
         <v>22</v>
       </c>
       <c r="C14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1197,19 +1197,19 @@
         <v>31</v>
       </c>
       <c r="C15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1217,19 +1217,19 @@
         <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1240,19 +1240,19 @@
         <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1263,16 +1263,16 @@
         <v>33</v>
       </c>
       <c r="C18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1283,19 +1283,19 @@
         <v>34</v>
       </c>
       <c r="C19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F19" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G19" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1303,19 +1303,19 @@
         <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1326,19 +1326,19 @@
         <v>35</v>
       </c>
       <c r="C21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F21" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1349,50 +1349,50 @@
         <v>36</v>
       </c>
       <c r="C22" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>111</v>
+      </c>
+      <c r="B23" t="s">
         <v>112</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>113</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>114</v>
       </c>
-      <c r="D23" t="s">
-        <v>115</v>
-      </c>
       <c r="E23" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>117</v>
+      </c>
+      <c r="B24" t="s">
+        <v>115</v>
+      </c>
+      <c r="C24" t="s">
+        <v>120</v>
+      </c>
+      <c r="D24" t="s">
         <v>118</v>
       </c>
-      <c r="B24" t="s">
-        <v>116</v>
-      </c>
-      <c r="C24" t="s">
-        <v>121</v>
-      </c>
-      <c r="D24" t="s">
-        <v>119</v>
-      </c>
       <c r="E24" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1403,30 +1403,30 @@
         <v>7</v>
       </c>
       <c r="C25" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D25" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E25" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B26" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C26" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D26" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -1446,10 +1446,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" t="s">
         <v>57</v>
-      </c>
-      <c r="B1" t="s">
-        <v>58</v>
       </c>
       <c r="C1" t="s">
         <v>38</v>
@@ -1457,35 +1457,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" t="s">
         <v>75</v>
       </c>
-      <c r="B2" t="s">
-        <v>76</v>
-      </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1496,7 +1496,7 @@
         <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1507,7 +1507,7 @@
         <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1518,7 +1518,7 @@
         <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1526,10 +1526,10 @@
         <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1537,10 +1537,10 @@
         <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1548,10 +1548,10 @@
         <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>